<commit_message>
Fix Shopify Product Category taxonomy compliance (100% valid) and document taxonomy standards in shopify-catalog-ops skill
</commit_message>
<xml_diff>
--- a/WinBachat_AA_Dot_Store_Review_and_Audit.xlsx
+++ b/WinBachat_AA_Dot_Store_Review_and_Audit.xlsx
@@ -486,7 +486,7 @@
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="45" customWidth="1" min="4" max="4"/>
     <col width="45" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
@@ -699,7 +699,7 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Cosmetics</t>
+          <t>Skin Care</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
@@ -864,7 +864,7 @@
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
@@ -919,7 +919,7 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>Cosmetics</t>
+          <t>Skin Care</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
@@ -974,7 +974,7 @@
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>Cosmetics</t>
+          <t>Skin Care</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
@@ -2019,7 +2019,7 @@
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>Baby Care</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
@@ -2074,7 +2074,7 @@
       </c>
       <c r="F29" s="7" t="inlineStr">
         <is>
-          <t>Baby Care</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G29" s="7" t="inlineStr">
@@ -2129,7 +2129,7 @@
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>Baby Care</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
@@ -2184,7 +2184,7 @@
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>Baby Care</t>
+          <t>Skin Care</t>
         </is>
       </c>
       <c r="G31" s="7" t="inlineStr">
@@ -2239,7 +2239,7 @@
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>Baby Care</t>
+          <t>Skin Care</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
@@ -2294,7 +2294,7 @@
       </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
-          <t>Baby Care</t>
+          <t>Skin Care</t>
         </is>
       </c>
       <c r="G33" s="7" t="inlineStr">
@@ -2349,7 +2349,7 @@
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>Baby Care</t>
+          <t>Skin Care</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
@@ -2404,7 +2404,7 @@
       </c>
       <c r="F35" s="7" t="inlineStr">
         <is>
-          <t>Baby Care</t>
+          <t>Skin Care</t>
         </is>
       </c>
       <c r="G35" s="7" t="inlineStr">
@@ -2459,7 +2459,7 @@
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>Baby Care</t>
+          <t>Skin Care</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
@@ -2514,7 +2514,7 @@
       </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
-          <t>Baby Care</t>
+          <t>Skin Care</t>
         </is>
       </c>
       <c r="G37" s="7" t="inlineStr">
@@ -2569,7 +2569,7 @@
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>Baby Care</t>
+          <t>Skin Care</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
@@ -2624,7 +2624,7 @@
       </c>
       <c r="F39" s="7" t="inlineStr">
         <is>
-          <t>Baby Care</t>
+          <t>Skin Care</t>
         </is>
       </c>
       <c r="G39" s="7" t="inlineStr">
@@ -2679,7 +2679,7 @@
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>Baby Care</t>
+          <t>Skin Care</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr">
@@ -2734,7 +2734,7 @@
       </c>
       <c r="F41" s="7" t="inlineStr">
         <is>
-          <t>Baby Care</t>
+          <t>Skin Care</t>
         </is>
       </c>
       <c r="G41" s="7" t="inlineStr">
@@ -2789,7 +2789,7 @@
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>Baby Care</t>
+          <t>Skin Care</t>
         </is>
       </c>
       <c r="G42" s="4" t="inlineStr">
@@ -2844,7 +2844,7 @@
       </c>
       <c r="F43" s="7" t="inlineStr">
         <is>
-          <t>Baby Care</t>
+          <t>Skin Care</t>
         </is>
       </c>
       <c r="G43" s="7" t="inlineStr">
@@ -2899,7 +2899,7 @@
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>Baby Care</t>
+          <t>Skin Care</t>
         </is>
       </c>
       <c r="G44" s="4" t="inlineStr">
@@ -2954,7 +2954,7 @@
       </c>
       <c r="F45" s="7" t="inlineStr">
         <is>
-          <t>Baby Care</t>
+          <t>Skin Care</t>
         </is>
       </c>
       <c r="G45" s="7" t="inlineStr">
@@ -3009,7 +3009,7 @@
       </c>
       <c r="F46" s="4" t="inlineStr">
         <is>
-          <t>Baby Care</t>
+          <t>Skin Care</t>
         </is>
       </c>
       <c r="G46" s="4" t="inlineStr">
@@ -3064,7 +3064,7 @@
       </c>
       <c r="F47" s="7" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G47" s="7" t="inlineStr">
@@ -3119,7 +3119,7 @@
       </c>
       <c r="F48" s="4" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G48" s="4" t="inlineStr">
@@ -3174,7 +3174,7 @@
       </c>
       <c r="F49" s="7" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G49" s="7" t="inlineStr">
@@ -3229,7 +3229,7 @@
       </c>
       <c r="F50" s="4" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G50" s="4" t="inlineStr">
@@ -3284,7 +3284,7 @@
       </c>
       <c r="F51" s="7" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G51" s="7" t="inlineStr">
@@ -3339,7 +3339,7 @@
       </c>
       <c r="F52" s="4" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G52" s="4" t="inlineStr">
@@ -3394,7 +3394,7 @@
       </c>
       <c r="F53" s="7" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G53" s="7" t="inlineStr">
@@ -3449,7 +3449,7 @@
       </c>
       <c r="F54" s="4" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G54" s="4" t="inlineStr">
@@ -3504,7 +3504,7 @@
       </c>
       <c r="F55" s="7" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G55" s="7" t="inlineStr">
@@ -3559,7 +3559,7 @@
       </c>
       <c r="F56" s="4" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G56" s="4" t="inlineStr">
@@ -3614,7 +3614,7 @@
       </c>
       <c r="F57" s="7" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G57" s="7" t="inlineStr">
@@ -3669,7 +3669,7 @@
       </c>
       <c r="F58" s="4" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G58" s="4" t="inlineStr">
@@ -3724,7 +3724,7 @@
       </c>
       <c r="F59" s="7" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G59" s="7" t="inlineStr">
@@ -3779,7 +3779,7 @@
       </c>
       <c r="F60" s="4" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G60" s="4" t="inlineStr">
@@ -3834,7 +3834,7 @@
       </c>
       <c r="F61" s="7" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G61" s="7" t="inlineStr">
@@ -3889,7 +3889,7 @@
       </c>
       <c r="F62" s="4" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G62" s="4" t="inlineStr">
@@ -3944,7 +3944,7 @@
       </c>
       <c r="F63" s="7" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G63" s="7" t="inlineStr">
@@ -3999,7 +3999,7 @@
       </c>
       <c r="F64" s="4" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G64" s="4" t="inlineStr">
@@ -4054,7 +4054,7 @@
       </c>
       <c r="F65" s="7" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G65" s="7" t="inlineStr">
@@ -4109,7 +4109,7 @@
       </c>
       <c r="F66" s="4" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G66" s="4" t="inlineStr">
@@ -4164,7 +4164,7 @@
       </c>
       <c r="F67" s="7" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G67" s="7" t="inlineStr">
@@ -4219,7 +4219,7 @@
       </c>
       <c r="F68" s="4" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G68" s="4" t="inlineStr">
@@ -4274,7 +4274,7 @@
       </c>
       <c r="F69" s="7" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G69" s="7" t="inlineStr">
@@ -4329,7 +4329,7 @@
       </c>
       <c r="F70" s="4" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G70" s="4" t="inlineStr">
@@ -4384,7 +4384,7 @@
       </c>
       <c r="F71" s="7" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G71" s="7" t="inlineStr">
@@ -4439,7 +4439,7 @@
       </c>
       <c r="F72" s="4" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G72" s="4" t="inlineStr">
@@ -4494,7 +4494,7 @@
       </c>
       <c r="F73" s="7" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G73" s="7" t="inlineStr">
@@ -4549,7 +4549,7 @@
       </c>
       <c r="F74" s="4" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G74" s="4" t="inlineStr">
@@ -4604,7 +4604,7 @@
       </c>
       <c r="F75" s="7" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G75" s="7" t="inlineStr">
@@ -4659,7 +4659,7 @@
       </c>
       <c r="F76" s="4" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G76" s="4" t="inlineStr">
@@ -4714,7 +4714,7 @@
       </c>
       <c r="F77" s="7" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G77" s="7" t="inlineStr">
@@ -4769,7 +4769,7 @@
       </c>
       <c r="F78" s="4" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G78" s="4" t="inlineStr">
@@ -4824,7 +4824,7 @@
       </c>
       <c r="F79" s="7" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G79" s="7" t="inlineStr">
@@ -4879,7 +4879,7 @@
       </c>
       <c r="F80" s="4" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G80" s="4" t="inlineStr">
@@ -4934,7 +4934,7 @@
       </c>
       <c r="F81" s="7" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G81" s="7" t="inlineStr">
@@ -4989,7 +4989,7 @@
       </c>
       <c r="F82" s="4" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G82" s="4" t="inlineStr">
@@ -5044,7 +5044,7 @@
       </c>
       <c r="F83" s="7" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G83" s="7" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="F84" s="4" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G84" s="4" t="inlineStr">
@@ -5154,7 +5154,7 @@
       </c>
       <c r="F85" s="7" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G85" s="7" t="inlineStr">
@@ -5209,7 +5209,7 @@
       </c>
       <c r="F86" s="4" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G86" s="4" t="inlineStr">
@@ -5264,7 +5264,7 @@
       </c>
       <c r="F87" s="7" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G87" s="7" t="inlineStr">
@@ -5319,7 +5319,7 @@
       </c>
       <c r="F88" s="4" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G88" s="4" t="inlineStr">
@@ -5374,7 +5374,7 @@
       </c>
       <c r="F89" s="7" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G89" s="7" t="inlineStr">
@@ -5429,7 +5429,7 @@
       </c>
       <c r="F90" s="4" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G90" s="4" t="inlineStr">
@@ -5484,7 +5484,7 @@
       </c>
       <c r="F91" s="7" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G91" s="7" t="inlineStr">
@@ -5539,7 +5539,7 @@
       </c>
       <c r="F92" s="4" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G92" s="4" t="inlineStr">
@@ -5594,7 +5594,7 @@
       </c>
       <c r="F93" s="7" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G93" s="7" t="inlineStr">
@@ -5649,7 +5649,7 @@
       </c>
       <c r="F94" s="4" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G94" s="4" t="inlineStr">
@@ -5704,7 +5704,7 @@
       </c>
       <c r="F95" s="7" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G95" s="7" t="inlineStr">
@@ -5759,7 +5759,7 @@
       </c>
       <c r="F96" s="4" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G96" s="4" t="inlineStr">
@@ -5814,7 +5814,7 @@
       </c>
       <c r="F97" s="7" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G97" s="7" t="inlineStr">
@@ -5869,7 +5869,7 @@
       </c>
       <c r="F98" s="4" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G98" s="4" t="inlineStr">
@@ -5924,7 +5924,7 @@
       </c>
       <c r="F99" s="7" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G99" s="7" t="inlineStr">
@@ -5979,7 +5979,7 @@
       </c>
       <c r="F100" s="4" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G100" s="4" t="inlineStr">
@@ -6034,7 +6034,7 @@
       </c>
       <c r="F101" s="7" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G101" s="7" t="inlineStr">
@@ -6089,7 +6089,7 @@
       </c>
       <c r="F102" s="4" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G102" s="4" t="inlineStr">
@@ -6144,7 +6144,7 @@
       </c>
       <c r="F103" s="7" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G103" s="7" t="inlineStr">
@@ -6199,7 +6199,7 @@
       </c>
       <c r="F104" s="4" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G104" s="4" t="inlineStr">
@@ -6254,7 +6254,7 @@
       </c>
       <c r="F105" s="7" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G105" s="7" t="inlineStr">
@@ -6309,7 +6309,7 @@
       </c>
       <c r="F106" s="4" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G106" s="4" t="inlineStr">
@@ -6364,7 +6364,7 @@
       </c>
       <c r="F107" s="7" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G107" s="7" t="inlineStr">
@@ -6419,7 +6419,7 @@
       </c>
       <c r="F108" s="4" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G108" s="4" t="inlineStr">
@@ -6474,7 +6474,7 @@
       </c>
       <c r="F109" s="7" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G109" s="7" t="inlineStr">
@@ -6529,7 +6529,7 @@
       </c>
       <c r="F110" s="4" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G110" s="4" t="inlineStr">
@@ -6584,7 +6584,7 @@
       </c>
       <c r="F111" s="7" t="inlineStr">
         <is>
-          <t>Fragrances</t>
+          <t>Perfumes &amp; Colognes</t>
         </is>
       </c>
       <c r="G111" s="7" t="inlineStr">

</xml_diff>

<commit_message>
Document shared group photos policy in AA Dot Store client review audit log
</commit_message>
<xml_diff>
--- a/WinBachat_AA_Dot_Store_Review_and_Audit.xlsx
+++ b/WinBachat_AA_Dot_Store_Review_and_Audit.xlsx
@@ -6624,12 +6624,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="45" customWidth="1" min="1" max="1"/>
     <col width="38" customWidth="1" min="2" max="2"/>
-    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
   </cols>
@@ -6877,6 +6877,114 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>Dorall Perfumes (A Art 29, 26 items)</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Shared Group Photos Only</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>26 scents listed; 7 group photos on disk (no individual bottle shots)</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>Published Active as individual listings with shared group gallery</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>Per store owner policy: kept active while awaiting client individual pack shots</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>Guys Body Spray (A Art 30, 8 items)</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>Shared Group Photos Only</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>8 fragrances listed; 1 group photo on disk</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="inlineStr">
+        <is>
+          <t>Published Active as individual listings with shared group photo</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="inlineStr">
+        <is>
+          <t>Per store owner policy: kept active with shared group shot</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>Kliock Perfumes (A Art 26, 6 items)</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>Shared Group Photos Only</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>6 scents listed; 1 group photo on disk</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>Published Active as individual listings with shared group photo</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>Per store owner policy: kept active with shared group shot</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>Inertia Perfumes (A Art 27 &amp; 28, 25 items)</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>Shared Group Photos Only</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>25 scents listed; 5 group photos on disk</t>
+        </is>
+      </c>
+      <c r="D13" s="10" t="inlineStr">
+        <is>
+          <t>Published Active as individual listings with shared group photos</t>
+        </is>
+      </c>
+      <c r="E13" s="10" t="inlineStr">
+        <is>
+          <t>Per store owner policy: kept active with shared group shots</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>